<commit_message>
OTP 2026.09 and CIViC 20260927
</commit_message>
<xml_diff>
--- a/data-raw/metadata_pharm_oncox.xlsx
+++ b/data-raw/metadata_pharm_oncox.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sigven/project_data/packages/package__pharmOncoX/pharmOncoX/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00FFD2DA-EF72-B441-951D-A64BA7C9C1F3}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{041D884E-7932-774B-8583-FF91C0140039}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5160" yWindow="1620" windowWidth="35840" windowHeight="19820" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
+    <workbookView xWindow="0" yWindow="1620" windowWidth="35840" windowHeight="19820" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
   </bookViews>
   <sheets>
     <sheet name="compounds" sheetId="2" r:id="rId1"/>
@@ -211,13 +211,13 @@
     <t>v2026</t>
   </si>
   <si>
-    <t>2026.06</t>
-  </si>
-  <si>
     <t>v20260715</t>
   </si>
   <si>
     <t>26.08e</t>
+  </si>
+  <si>
+    <t>2026.09</t>
   </si>
 </sst>
 </file>
@@ -681,7 +681,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
@@ -707,7 +707,7 @@
         <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F3" t="s">
         <v>9</v>
@@ -835,7 +835,7 @@
         <v>18</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
updated NCI Thesaurus and CIViC
</commit_message>
<xml_diff>
--- a/data-raw/metadata_pharm_oncox.xlsx
+++ b/data-raw/metadata_pharm_oncox.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sigven/project_data/packages/package__pharmOncoX/pharmOncoX/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{041D884E-7932-774B-8583-FF91C0140039}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BA738FC-8C14-CA4B-A3FD-F00C1DE87188}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1620" windowWidth="35840" windowHeight="19820" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
+    <workbookView xWindow="0" yWindow="1620" windowWidth="35840" windowHeight="19820" activeTab="1" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
   </bookViews>
   <sheets>
     <sheet name="compounds" sheetId="2" r:id="rId1"/>
@@ -214,10 +214,10 @@
     <t>v20260715</t>
   </si>
   <si>
-    <t>26.08e</t>
-  </si>
-  <si>
     <t>2026.09</t>
+  </si>
+  <si>
+    <t>26.09d</t>
   </si>
 </sst>
 </file>
@@ -681,7 +681,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
@@ -707,7 +707,7 @@
         <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F3" t="s">
         <v>9</v>

</xml_diff>